<commit_message>
fix(#298): tableau des 4 statuts RNIV dans intro pagecontent du ValueSet
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com> 6efa8b822e4ea0a0215105e66bc3a4c8062a07f9
</commit_message>
<xml_diff>
--- a/fix/issue-298-identity-status-rniv/ig/ValueSet-fr-core-vs-identity-reliability-ins-status.xlsx
+++ b/fix/issue-298-identity-status-rniv/ig/ValueSet-fr-core-vs-identity-reliability-ins-status.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-05T12:16:59+00:00</t>
+    <t>2026-06-05T12:18:27+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -87,13 +87,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Les 4 statuts de confiance de l'identité définis par le RNIV [EXI SI 07]. Ces statuts sont exclusifs les uns des autres.
-| Code | Statut RNIV | INSi (I) | Contrôle (C) |
-|---|---|---|---|
-| PROV | Identité provisoire | − | − |
-| RECUP | Identité récupérée | + | − |
-| VALI | Identité validée | − | + |
-| QUAL | Identité qualifiée | + | + |</t>
+    <t>Les 4 statuts de confiance de l'identité définis par le RNIV [EXI SI 07]. Ces statuts sont exclusifs les uns des autres.</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>